<commit_message>
test(7762): CT-RAP-002 APROVADO no modulo Internacional - 160 divergencias viraram 0
Build V 1.0.260804.2007, ref 07/2026, script ct_rap_tipo_apolice_reteste.py:
  495 linhas · 464 conferidas contra tb_apo_int_cit.e_avb
  DIARIA indevida (#7975): 0     rotulo divergente do cadastro (#8008): 0 (eram 160)

Nota de metodo registrada no plano: a rodada do Gestao com filtro tipoRamo=INTERNACIONAL
NAO conta como este CT - e outra tela. Ela entra como 2a medicao do CT-RAP-003. Aproveitar
repetiria o erro que reabriu o card: aprovar com medicao que nao corresponde ao CT.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sprint-11-citweb/pbi-7762/evidencias/CT-RAP-RETESTE-7975/Analitico-Producao-Int-07-2026.xlsx
+++ b/docs/sprint-11-citweb/pbi-7762/evidencias/CT-RAP-RETESTE-7975/Analitico-Producao-Int-07-2026.xlsx
@@ -26,7 +26,7 @@
     <t>CRITÉRIO DE SELEÇÃO: TUDO</t>
   </si>
   <si>
-    <t>Gerado em 04/08/2026 10:36</t>
+    <t>Gerado em 05/08/2026 10:39</t>
   </si>
   <si>
     <t>Ano/Mês Refer</t>
@@ -197,7 +197,7 @@
     <t>CITNET</t>
   </si>
   <si>
-    <t>MENSAL DET</t>
+    <t>AVERBÁVEL</t>
   </si>
   <si>
     <t xml:space="preserve">4TECH MAQUINAS E EQUIPAMENTOS LTDA                                                                  </t>
@@ -293,10 +293,10 @@
     <t>ANDREIA</t>
   </si>
   <si>
-    <t>6.029.924.709,24</t>
-  </si>
-  <si>
-    <t>21.501.024,17</t>
+    <t>6.035.534.194,27</t>
+  </si>
+  <si>
+    <t>21.521.024,17</t>
   </si>
   <si>
     <t>DIÁRIA</t>

</xml_diff>